<commit_message>
arr-check: the ARR bridge, three ways (bridge.csv, bridge_accounts.csv, Bridge sheet, report section)
Schedule, invoices and supported bases from the same customer months,
a difference row, and the accounts behind every movement. Identity
asserted every month. On the Larkspur set the planted Lantern Field
churn shows on the schedule basis in 2025-09 and not on the invoices
basis, because billing continues. Five key files byte identical; both
receipts verify. Started by Codex on codex/cx-067-bridge, finished here.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015rgfqU3HzoKDqHvRpr81av
</commit_message>
<xml_diff>
--- a/example/outputs/pilot.xlsx
+++ b/example/outputs/pilot.xlsx
@@ -14,6 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cohorts" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Match" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Customer month" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bridge" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -41475,4 +41476,1649 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I49"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>month</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>basis</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>start</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>reactivation</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>expansion</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>contraction</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>churn</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>end</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2024-11</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>difference</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>6700</v>
+      </c>
+      <c r="D2" t="n">
+        <v>-3800</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="n">
+        <v>2900</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2024-11</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>invoices</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>69400</v>
+      </c>
+      <c r="D3" t="n">
+        <v>3800</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="n">
+        <v>73200</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2024-11</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>schedule</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>75800</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="n">
+        <v>75800</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2024-11</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>supported</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>69100</v>
+      </c>
+      <c r="D5" t="n">
+        <v>3800</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
+        <v>72900</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2024-12</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>difference</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>2900</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="n">
+        <v>2900</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2024-12</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>invoices</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>73200</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" t="n">
+        <v>73200</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2024-12</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>schedule</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>75800</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" t="n">
+        <v>75800</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2024-12</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>supported</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>72900</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" t="n">
+        <v>72900</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>difference</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>2900</v>
+      </c>
+      <c r="D10" t="n">
+        <v>4000</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" t="n">
+        <v>6900</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>invoices</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>73200</v>
+      </c>
+      <c r="D11" t="n">
+        <v>4000</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" t="n">
+        <v>77200</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>schedule</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>75800</v>
+      </c>
+      <c r="D12" t="n">
+        <v>8000</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" t="n">
+        <v>83800</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>supported</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>72900</v>
+      </c>
+      <c r="D13" t="n">
+        <v>4000</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" t="n">
+        <v>76900</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2025-02</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>difference</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>6900</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" t="n">
+        <v>6900</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2025-02</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>invoices</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>77200</v>
+      </c>
+      <c r="D15" t="n">
+        <v>950</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" t="n">
+        <v>78150</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2025-02</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>schedule</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>83800</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" t="n">
+        <v>83800</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2025-02</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>supported</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>76900</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" t="n">
+        <v>76900</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>difference</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>6900</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" t="n">
+        <v>6900</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>invoices</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>78150</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" t="n">
+        <v>78150</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>schedule</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>83800</v>
+      </c>
+      <c r="D20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" t="n">
+        <v>0</v>
+      </c>
+      <c r="I20" t="n">
+        <v>83800</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>supported</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>76900</v>
+      </c>
+      <c r="D21" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I21" t="n">
+        <v>76900</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2025-04</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>difference</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>6900</v>
+      </c>
+      <c r="D22" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" t="n">
+        <v>-4000</v>
+      </c>
+      <c r="G22" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" t="n">
+        <v>0</v>
+      </c>
+      <c r="I22" t="n">
+        <v>2900</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2025-04</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>invoices</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>78150</v>
+      </c>
+      <c r="D23" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" t="n">
+        <v>5700</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" t="n">
+        <v>4000</v>
+      </c>
+      <c r="I23" t="n">
+        <v>79850</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2025-04</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>schedule</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>83800</v>
+      </c>
+      <c r="D24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" t="n">
+        <v>4000</v>
+      </c>
+      <c r="I24" t="n">
+        <v>79800</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2025-04</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>supported</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>76900</v>
+      </c>
+      <c r="D25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" t="n">
+        <v>4000</v>
+      </c>
+      <c r="G25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" t="n">
+        <v>4000</v>
+      </c>
+      <c r="I25" t="n">
+        <v>76900</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2025-05</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>difference</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>2900</v>
+      </c>
+      <c r="D26" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" t="n">
+        <v>0</v>
+      </c>
+      <c r="I26" t="n">
+        <v>2900</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2025-05</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>invoices</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>79850</v>
+      </c>
+      <c r="D27" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" t="n">
+        <v>1700</v>
+      </c>
+      <c r="H27" t="n">
+        <v>0</v>
+      </c>
+      <c r="I27" t="n">
+        <v>78150</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2025-05</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>schedule</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>79800</v>
+      </c>
+      <c r="D28" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" t="n">
+        <v>600</v>
+      </c>
+      <c r="G28" t="n">
+        <v>0</v>
+      </c>
+      <c r="H28" t="n">
+        <v>0</v>
+      </c>
+      <c r="I28" t="n">
+        <v>80400</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2025-05</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>supported</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>76900</v>
+      </c>
+      <c r="D29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" t="n">
+        <v>600</v>
+      </c>
+      <c r="G29" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" t="n">
+        <v>0</v>
+      </c>
+      <c r="I29" t="n">
+        <v>77500</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2025-06</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>difference</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>2900</v>
+      </c>
+      <c r="D30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" t="n">
+        <v>0</v>
+      </c>
+      <c r="I30" t="n">
+        <v>2900</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2025-06</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>invoices</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>78150</v>
+      </c>
+      <c r="D31" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" t="n">
+        <v>600</v>
+      </c>
+      <c r="G31" t="n">
+        <v>400</v>
+      </c>
+      <c r="H31" t="n">
+        <v>3100</v>
+      </c>
+      <c r="I31" t="n">
+        <v>75250</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2025-06</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>schedule</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>80400</v>
+      </c>
+      <c r="D32" t="n">
+        <v>0</v>
+      </c>
+      <c r="E32" t="n">
+        <v>0</v>
+      </c>
+      <c r="F32" t="n">
+        <v>0</v>
+      </c>
+      <c r="G32" t="n">
+        <v>400</v>
+      </c>
+      <c r="H32" t="n">
+        <v>3100</v>
+      </c>
+      <c r="I32" t="n">
+        <v>76900</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2025-06</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>supported</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>77500</v>
+      </c>
+      <c r="D33" t="n">
+        <v>0</v>
+      </c>
+      <c r="E33" t="n">
+        <v>0</v>
+      </c>
+      <c r="F33" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" t="n">
+        <v>400</v>
+      </c>
+      <c r="H33" t="n">
+        <v>3100</v>
+      </c>
+      <c r="I33" t="n">
+        <v>74000</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2025-07</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>difference</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>2900</v>
+      </c>
+      <c r="D34" t="n">
+        <v>0</v>
+      </c>
+      <c r="E34" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" t="n">
+        <v>0</v>
+      </c>
+      <c r="G34" t="n">
+        <v>0</v>
+      </c>
+      <c r="H34" t="n">
+        <v>0</v>
+      </c>
+      <c r="I34" t="n">
+        <v>2900</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2025-07</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>invoices</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>75250</v>
+      </c>
+      <c r="D35" t="n">
+        <v>0</v>
+      </c>
+      <c r="E35" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" t="n">
+        <v>0</v>
+      </c>
+      <c r="G35" t="n">
+        <v>0</v>
+      </c>
+      <c r="H35" t="n">
+        <v>3100</v>
+      </c>
+      <c r="I35" t="n">
+        <v>72150</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2025-07</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>schedule</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>76900</v>
+      </c>
+      <c r="D36" t="n">
+        <v>0</v>
+      </c>
+      <c r="E36" t="n">
+        <v>0</v>
+      </c>
+      <c r="F36" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" t="n">
+        <v>0</v>
+      </c>
+      <c r="H36" t="n">
+        <v>3100</v>
+      </c>
+      <c r="I36" t="n">
+        <v>73800</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2025-07</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>supported</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>74000</v>
+      </c>
+      <c r="D37" t="n">
+        <v>0</v>
+      </c>
+      <c r="E37" t="n">
+        <v>0</v>
+      </c>
+      <c r="F37" t="n">
+        <v>0</v>
+      </c>
+      <c r="G37" t="n">
+        <v>0</v>
+      </c>
+      <c r="H37" t="n">
+        <v>3100</v>
+      </c>
+      <c r="I37" t="n">
+        <v>70900</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2025-08</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>difference</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>2900</v>
+      </c>
+      <c r="D38" t="n">
+        <v>0</v>
+      </c>
+      <c r="E38" t="n">
+        <v>0</v>
+      </c>
+      <c r="F38" t="n">
+        <v>0</v>
+      </c>
+      <c r="G38" t="n">
+        <v>0</v>
+      </c>
+      <c r="H38" t="n">
+        <v>0</v>
+      </c>
+      <c r="I38" t="n">
+        <v>2900</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2025-08</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>invoices</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>72150</v>
+      </c>
+      <c r="D39" t="n">
+        <v>0</v>
+      </c>
+      <c r="E39" t="n">
+        <v>0</v>
+      </c>
+      <c r="F39" t="n">
+        <v>0</v>
+      </c>
+      <c r="G39" t="n">
+        <v>0</v>
+      </c>
+      <c r="H39" t="n">
+        <v>0</v>
+      </c>
+      <c r="I39" t="n">
+        <v>72150</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2025-08</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>schedule</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>73800</v>
+      </c>
+      <c r="D40" t="n">
+        <v>0</v>
+      </c>
+      <c r="E40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F40" t="n">
+        <v>0</v>
+      </c>
+      <c r="G40" t="n">
+        <v>0</v>
+      </c>
+      <c r="H40" t="n">
+        <v>0</v>
+      </c>
+      <c r="I40" t="n">
+        <v>73800</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2025-08</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>supported</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>70900</v>
+      </c>
+      <c r="D41" t="n">
+        <v>0</v>
+      </c>
+      <c r="E41" t="n">
+        <v>0</v>
+      </c>
+      <c r="F41" t="n">
+        <v>0</v>
+      </c>
+      <c r="G41" t="n">
+        <v>0</v>
+      </c>
+      <c r="H41" t="n">
+        <v>0</v>
+      </c>
+      <c r="I41" t="n">
+        <v>70900</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2025-09</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>difference</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>2900</v>
+      </c>
+      <c r="D42" t="n">
+        <v>0</v>
+      </c>
+      <c r="E42" t="n">
+        <v>0</v>
+      </c>
+      <c r="F42" t="n">
+        <v>0</v>
+      </c>
+      <c r="G42" t="n">
+        <v>0</v>
+      </c>
+      <c r="H42" t="n">
+        <v>0</v>
+      </c>
+      <c r="I42" t="n">
+        <v>2900</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2025-09</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>invoices</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>72150</v>
+      </c>
+      <c r="D43" t="n">
+        <v>0</v>
+      </c>
+      <c r="E43" t="n">
+        <v>0</v>
+      </c>
+      <c r="F43" t="n">
+        <v>0</v>
+      </c>
+      <c r="G43" t="n">
+        <v>0</v>
+      </c>
+      <c r="H43" t="n">
+        <v>0</v>
+      </c>
+      <c r="I43" t="n">
+        <v>72150</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2025-09</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>schedule</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>73800</v>
+      </c>
+      <c r="D44" t="n">
+        <v>0</v>
+      </c>
+      <c r="E44" t="n">
+        <v>0</v>
+      </c>
+      <c r="F44" t="n">
+        <v>0</v>
+      </c>
+      <c r="G44" t="n">
+        <v>0</v>
+      </c>
+      <c r="H44" t="n">
+        <v>1400</v>
+      </c>
+      <c r="I44" t="n">
+        <v>72400</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2025-09</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>supported</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>70900</v>
+      </c>
+      <c r="D45" t="n">
+        <v>0</v>
+      </c>
+      <c r="E45" t="n">
+        <v>0</v>
+      </c>
+      <c r="F45" t="n">
+        <v>0</v>
+      </c>
+      <c r="G45" t="n">
+        <v>0</v>
+      </c>
+      <c r="H45" t="n">
+        <v>1400</v>
+      </c>
+      <c r="I45" t="n">
+        <v>69500</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2025-10</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>difference</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>2900</v>
+      </c>
+      <c r="D46" t="n">
+        <v>0</v>
+      </c>
+      <c r="E46" t="n">
+        <v>0</v>
+      </c>
+      <c r="F46" t="n">
+        <v>0</v>
+      </c>
+      <c r="G46" t="n">
+        <v>0</v>
+      </c>
+      <c r="H46" t="n">
+        <v>0</v>
+      </c>
+      <c r="I46" t="n">
+        <v>2900</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2025-10</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>invoices</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>72150</v>
+      </c>
+      <c r="D47" t="n">
+        <v>0</v>
+      </c>
+      <c r="E47" t="n">
+        <v>0</v>
+      </c>
+      <c r="F47" t="n">
+        <v>0</v>
+      </c>
+      <c r="G47" t="n">
+        <v>0</v>
+      </c>
+      <c r="H47" t="n">
+        <v>0</v>
+      </c>
+      <c r="I47" t="n">
+        <v>72150</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2025-10</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>schedule</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>72400</v>
+      </c>
+      <c r="D48" t="n">
+        <v>0</v>
+      </c>
+      <c r="E48" t="n">
+        <v>0</v>
+      </c>
+      <c r="F48" t="n">
+        <v>0</v>
+      </c>
+      <c r="G48" t="n">
+        <v>0</v>
+      </c>
+      <c r="H48" t="n">
+        <v>0</v>
+      </c>
+      <c r="I48" t="n">
+        <v>72400</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2025-10</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>supported</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>69500</v>
+      </c>
+      <c r="D49" t="n">
+        <v>0</v>
+      </c>
+      <c r="E49" t="n">
+        <v>0</v>
+      </c>
+      <c r="F49" t="n">
+        <v>0</v>
+      </c>
+      <c r="G49" t="n">
+        <v>0</v>
+      </c>
+      <c r="H49" t="n">
+        <v>0</v>
+      </c>
+      <c r="I49" t="n">
+        <v>69500</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
arr-check: deferred revenue for QuickBooks Online, with a journal that ties
On top of Claude Code's deferred lane (rebased onto main with the bridge):
- periodless recurring lines get a service period only when the amount is
  an exact whole multiple of the schedule MRR, 2 to 36 months, marked
  period_source = inferred_from_schedule; anything else is not guessed
- journal.csv is the QuickBooks month end true up of the deferred balance
  per customer; monthly customers produce no line; ties to the roll
  forward every month
- example/quickbooks/ with a stated expected deferred balance of 49,300 at
  2025-10, reproduced account by account
- write_report carries the bridge, the answers and the deferred sections
Larkspur: five key files and the bridge unchanged in value; both receipts
verify.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015rgfqU3HzoKDqHvRpr81av
</commit_message>
<xml_diff>
--- a/example/outputs/pilot.xlsx
+++ b/example/outputs/pilot.xlsx
@@ -14,7 +14,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cohorts" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Match" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Customer month" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bridge" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deferred" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deferred by account" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bridge" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -478,6 +480,1651 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I49"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>month</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>basis</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>start</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>reactivation</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>expansion</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>contraction</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>churn</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>end</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2024-11</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>difference</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>6700</v>
+      </c>
+      <c r="D2" t="n">
+        <v>-3800</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="n">
+        <v>2900</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2024-11</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>invoices</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>69400</v>
+      </c>
+      <c r="D3" t="n">
+        <v>3800</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="n">
+        <v>73200</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2024-11</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>schedule</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>75800</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="n">
+        <v>75800</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2024-11</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>supported</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>69100</v>
+      </c>
+      <c r="D5" t="n">
+        <v>3800</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
+        <v>72900</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2024-12</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>difference</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>2900</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="n">
+        <v>2900</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2024-12</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>invoices</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>73200</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" t="n">
+        <v>73200</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2024-12</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>schedule</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>75800</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" t="n">
+        <v>75800</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2024-12</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>supported</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>72900</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" t="n">
+        <v>72900</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>difference</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>2900</v>
+      </c>
+      <c r="D10" t="n">
+        <v>4000</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" t="n">
+        <v>6900</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>invoices</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>73200</v>
+      </c>
+      <c r="D11" t="n">
+        <v>4000</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" t="n">
+        <v>77200</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>schedule</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>75800</v>
+      </c>
+      <c r="D12" t="n">
+        <v>8000</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" t="n">
+        <v>83800</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>supported</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>72900</v>
+      </c>
+      <c r="D13" t="n">
+        <v>4000</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" t="n">
+        <v>76900</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2025-02</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>difference</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>6900</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" t="n">
+        <v>6900</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2025-02</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>invoices</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>77200</v>
+      </c>
+      <c r="D15" t="n">
+        <v>950</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" t="n">
+        <v>78150</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2025-02</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>schedule</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>83800</v>
+      </c>
+      <c r="D16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" t="n">
+        <v>83800</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2025-02</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>supported</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>76900</v>
+      </c>
+      <c r="D17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" t="n">
+        <v>76900</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>difference</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>6900</v>
+      </c>
+      <c r="D18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" t="n">
+        <v>6900</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>invoices</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>78150</v>
+      </c>
+      <c r="D19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" t="n">
+        <v>78150</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>schedule</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>83800</v>
+      </c>
+      <c r="D20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" t="n">
+        <v>0</v>
+      </c>
+      <c r="I20" t="n">
+        <v>83800</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>supported</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>76900</v>
+      </c>
+      <c r="D21" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" t="n">
+        <v>0</v>
+      </c>
+      <c r="I21" t="n">
+        <v>76900</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2025-04</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>difference</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>6900</v>
+      </c>
+      <c r="D22" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" t="n">
+        <v>-4000</v>
+      </c>
+      <c r="G22" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" t="n">
+        <v>0</v>
+      </c>
+      <c r="I22" t="n">
+        <v>2900</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2025-04</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>invoices</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>78150</v>
+      </c>
+      <c r="D23" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" t="n">
+        <v>5700</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" t="n">
+        <v>4000</v>
+      </c>
+      <c r="I23" t="n">
+        <v>79850</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2025-04</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>schedule</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>83800</v>
+      </c>
+      <c r="D24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" t="n">
+        <v>4000</v>
+      </c>
+      <c r="I24" t="n">
+        <v>79800</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2025-04</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>supported</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>76900</v>
+      </c>
+      <c r="D25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" t="n">
+        <v>4000</v>
+      </c>
+      <c r="G25" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" t="n">
+        <v>4000</v>
+      </c>
+      <c r="I25" t="n">
+        <v>76900</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2025-05</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>difference</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>2900</v>
+      </c>
+      <c r="D26" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" t="n">
+        <v>0</v>
+      </c>
+      <c r="I26" t="n">
+        <v>2900</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2025-05</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>invoices</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>79850</v>
+      </c>
+      <c r="D27" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" t="n">
+        <v>1700</v>
+      </c>
+      <c r="H27" t="n">
+        <v>0</v>
+      </c>
+      <c r="I27" t="n">
+        <v>78150</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2025-05</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>schedule</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>79800</v>
+      </c>
+      <c r="D28" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" t="n">
+        <v>600</v>
+      </c>
+      <c r="G28" t="n">
+        <v>0</v>
+      </c>
+      <c r="H28" t="n">
+        <v>0</v>
+      </c>
+      <c r="I28" t="n">
+        <v>80400</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2025-05</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>supported</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>76900</v>
+      </c>
+      <c r="D29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" t="n">
+        <v>600</v>
+      </c>
+      <c r="G29" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" t="n">
+        <v>0</v>
+      </c>
+      <c r="I29" t="n">
+        <v>77500</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2025-06</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>difference</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>2900</v>
+      </c>
+      <c r="D30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" t="n">
+        <v>0</v>
+      </c>
+      <c r="I30" t="n">
+        <v>2900</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2025-06</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>invoices</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>78150</v>
+      </c>
+      <c r="D31" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" t="n">
+        <v>600</v>
+      </c>
+      <c r="G31" t="n">
+        <v>400</v>
+      </c>
+      <c r="H31" t="n">
+        <v>3100</v>
+      </c>
+      <c r="I31" t="n">
+        <v>75250</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2025-06</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>schedule</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>80400</v>
+      </c>
+      <c r="D32" t="n">
+        <v>0</v>
+      </c>
+      <c r="E32" t="n">
+        <v>0</v>
+      </c>
+      <c r="F32" t="n">
+        <v>0</v>
+      </c>
+      <c r="G32" t="n">
+        <v>400</v>
+      </c>
+      <c r="H32" t="n">
+        <v>3100</v>
+      </c>
+      <c r="I32" t="n">
+        <v>76900</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2025-06</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>supported</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>77500</v>
+      </c>
+      <c r="D33" t="n">
+        <v>0</v>
+      </c>
+      <c r="E33" t="n">
+        <v>0</v>
+      </c>
+      <c r="F33" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" t="n">
+        <v>400</v>
+      </c>
+      <c r="H33" t="n">
+        <v>3100</v>
+      </c>
+      <c r="I33" t="n">
+        <v>74000</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2025-07</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>difference</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>2900</v>
+      </c>
+      <c r="D34" t="n">
+        <v>0</v>
+      </c>
+      <c r="E34" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" t="n">
+        <v>0</v>
+      </c>
+      <c r="G34" t="n">
+        <v>0</v>
+      </c>
+      <c r="H34" t="n">
+        <v>0</v>
+      </c>
+      <c r="I34" t="n">
+        <v>2900</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2025-07</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>invoices</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>75250</v>
+      </c>
+      <c r="D35" t="n">
+        <v>0</v>
+      </c>
+      <c r="E35" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" t="n">
+        <v>0</v>
+      </c>
+      <c r="G35" t="n">
+        <v>0</v>
+      </c>
+      <c r="H35" t="n">
+        <v>3100</v>
+      </c>
+      <c r="I35" t="n">
+        <v>72150</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2025-07</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>schedule</t>
+        </is>
+      </c>
+      <c r="C36" t="n">
+        <v>76900</v>
+      </c>
+      <c r="D36" t="n">
+        <v>0</v>
+      </c>
+      <c r="E36" t="n">
+        <v>0</v>
+      </c>
+      <c r="F36" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" t="n">
+        <v>0</v>
+      </c>
+      <c r="H36" t="n">
+        <v>3100</v>
+      </c>
+      <c r="I36" t="n">
+        <v>73800</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2025-07</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>supported</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>74000</v>
+      </c>
+      <c r="D37" t="n">
+        <v>0</v>
+      </c>
+      <c r="E37" t="n">
+        <v>0</v>
+      </c>
+      <c r="F37" t="n">
+        <v>0</v>
+      </c>
+      <c r="G37" t="n">
+        <v>0</v>
+      </c>
+      <c r="H37" t="n">
+        <v>3100</v>
+      </c>
+      <c r="I37" t="n">
+        <v>70900</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2025-08</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>difference</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>2900</v>
+      </c>
+      <c r="D38" t="n">
+        <v>0</v>
+      </c>
+      <c r="E38" t="n">
+        <v>0</v>
+      </c>
+      <c r="F38" t="n">
+        <v>0</v>
+      </c>
+      <c r="G38" t="n">
+        <v>0</v>
+      </c>
+      <c r="H38" t="n">
+        <v>0</v>
+      </c>
+      <c r="I38" t="n">
+        <v>2900</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2025-08</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>invoices</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>72150</v>
+      </c>
+      <c r="D39" t="n">
+        <v>0</v>
+      </c>
+      <c r="E39" t="n">
+        <v>0</v>
+      </c>
+      <c r="F39" t="n">
+        <v>0</v>
+      </c>
+      <c r="G39" t="n">
+        <v>0</v>
+      </c>
+      <c r="H39" t="n">
+        <v>0</v>
+      </c>
+      <c r="I39" t="n">
+        <v>72150</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2025-08</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>schedule</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>73800</v>
+      </c>
+      <c r="D40" t="n">
+        <v>0</v>
+      </c>
+      <c r="E40" t="n">
+        <v>0</v>
+      </c>
+      <c r="F40" t="n">
+        <v>0</v>
+      </c>
+      <c r="G40" t="n">
+        <v>0</v>
+      </c>
+      <c r="H40" t="n">
+        <v>0</v>
+      </c>
+      <c r="I40" t="n">
+        <v>73800</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2025-08</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>supported</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>70900</v>
+      </c>
+      <c r="D41" t="n">
+        <v>0</v>
+      </c>
+      <c r="E41" t="n">
+        <v>0</v>
+      </c>
+      <c r="F41" t="n">
+        <v>0</v>
+      </c>
+      <c r="G41" t="n">
+        <v>0</v>
+      </c>
+      <c r="H41" t="n">
+        <v>0</v>
+      </c>
+      <c r="I41" t="n">
+        <v>70900</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2025-09</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>difference</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>2900</v>
+      </c>
+      <c r="D42" t="n">
+        <v>0</v>
+      </c>
+      <c r="E42" t="n">
+        <v>0</v>
+      </c>
+      <c r="F42" t="n">
+        <v>0</v>
+      </c>
+      <c r="G42" t="n">
+        <v>0</v>
+      </c>
+      <c r="H42" t="n">
+        <v>0</v>
+      </c>
+      <c r="I42" t="n">
+        <v>2900</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2025-09</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>invoices</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>72150</v>
+      </c>
+      <c r="D43" t="n">
+        <v>0</v>
+      </c>
+      <c r="E43" t="n">
+        <v>0</v>
+      </c>
+      <c r="F43" t="n">
+        <v>0</v>
+      </c>
+      <c r="G43" t="n">
+        <v>0</v>
+      </c>
+      <c r="H43" t="n">
+        <v>0</v>
+      </c>
+      <c r="I43" t="n">
+        <v>72150</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2025-09</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>schedule</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>73800</v>
+      </c>
+      <c r="D44" t="n">
+        <v>0</v>
+      </c>
+      <c r="E44" t="n">
+        <v>0</v>
+      </c>
+      <c r="F44" t="n">
+        <v>0</v>
+      </c>
+      <c r="G44" t="n">
+        <v>0</v>
+      </c>
+      <c r="H44" t="n">
+        <v>1400</v>
+      </c>
+      <c r="I44" t="n">
+        <v>72400</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2025-09</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>supported</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>70900</v>
+      </c>
+      <c r="D45" t="n">
+        <v>0</v>
+      </c>
+      <c r="E45" t="n">
+        <v>0</v>
+      </c>
+      <c r="F45" t="n">
+        <v>0</v>
+      </c>
+      <c r="G45" t="n">
+        <v>0</v>
+      </c>
+      <c r="H45" t="n">
+        <v>1400</v>
+      </c>
+      <c r="I45" t="n">
+        <v>69500</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2025-10</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>difference</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>2900</v>
+      </c>
+      <c r="D46" t="n">
+        <v>0</v>
+      </c>
+      <c r="E46" t="n">
+        <v>0</v>
+      </c>
+      <c r="F46" t="n">
+        <v>0</v>
+      </c>
+      <c r="G46" t="n">
+        <v>0</v>
+      </c>
+      <c r="H46" t="n">
+        <v>0</v>
+      </c>
+      <c r="I46" t="n">
+        <v>2900</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2025-10</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>invoices</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>72150</v>
+      </c>
+      <c r="D47" t="n">
+        <v>0</v>
+      </c>
+      <c r="E47" t="n">
+        <v>0</v>
+      </c>
+      <c r="F47" t="n">
+        <v>0</v>
+      </c>
+      <c r="G47" t="n">
+        <v>0</v>
+      </c>
+      <c r="H47" t="n">
+        <v>0</v>
+      </c>
+      <c r="I47" t="n">
+        <v>72150</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2025-10</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>schedule</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>72400</v>
+      </c>
+      <c r="D48" t="n">
+        <v>0</v>
+      </c>
+      <c r="E48" t="n">
+        <v>0</v>
+      </c>
+      <c r="F48" t="n">
+        <v>0</v>
+      </c>
+      <c r="G48" t="n">
+        <v>0</v>
+      </c>
+      <c r="H48" t="n">
+        <v>0</v>
+      </c>
+      <c r="I48" t="n">
+        <v>72400</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2025-10</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>supported</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>69500</v>
+      </c>
+      <c r="D49" t="n">
+        <v>0</v>
+      </c>
+      <c r="E49" t="n">
+        <v>0</v>
+      </c>
+      <c r="F49" t="n">
+        <v>0</v>
+      </c>
+      <c r="G49" t="n">
+        <v>0</v>
+      </c>
+      <c r="H49" t="n">
+        <v>0</v>
+      </c>
+      <c r="I49" t="n">
+        <v>69500</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -41484,7 +43131,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I49"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -41495,42 +43142,42 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>basis</t>
+          <t>opening</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>start</t>
+          <t>billings</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>new</t>
+          <t>recognised</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>reactivation</t>
+          <t>closing</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>expansion</t>
+          <t>closing_deferred</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>contraction</t>
+          <t>closing_unbilled</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>churn</t>
+          <t>gl_balance</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>end</t>
+          <t>difference</t>
         </is>
       </c>
     </row>
@@ -41540,1583 +43187,1210 @@
           <t>2024-11</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>difference</t>
-        </is>
+      <c r="B2" t="n">
+        <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>6700</v>
+        <v>95200</v>
       </c>
       <c r="D2" t="n">
-        <v>-3800</v>
+        <v>73200</v>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>22000</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>22000</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>0</v>
+        <v>22800</v>
       </c>
       <c r="I2" t="n">
-        <v>2900</v>
+        <v>-800</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2024-11</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>invoices</t>
-        </is>
+          <t>2024-12</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>22000</v>
       </c>
       <c r="C3" t="n">
-        <v>69400</v>
+        <v>71200</v>
       </c>
       <c r="D3" t="n">
-        <v>3800</v>
+        <v>73200</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>20000</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>20000</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>0</v>
+        <v>20800</v>
       </c>
       <c r="I3" t="n">
-        <v>73200</v>
+        <v>-800</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2024-11</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>schedule</t>
-        </is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>20000</v>
       </c>
       <c r="C4" t="n">
-        <v>75800</v>
+        <v>75200</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>77200</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>18000</v>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
+        <v>18000</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>0</v>
+        <v>18800</v>
       </c>
       <c r="I4" t="n">
-        <v>75800</v>
+        <v>-800</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2024-11</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>supported</t>
-        </is>
+          <t>2025-02</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>18000</v>
       </c>
       <c r="C5" t="n">
-        <v>69100</v>
+        <v>76150</v>
       </c>
       <c r="D5" t="n">
-        <v>3800</v>
+        <v>78150</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>16000</v>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>16000</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>0</v>
+        <v>16800</v>
       </c>
       <c r="I5" t="n">
-        <v>72900</v>
+        <v>-800</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2024-12</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>difference</t>
-        </is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>16000</v>
       </c>
       <c r="C6" t="n">
-        <v>2900</v>
+        <v>76150</v>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>78150</v>
       </c>
       <c r="E6" t="n">
-        <v>0</v>
+        <v>14000</v>
       </c>
       <c r="F6" t="n">
-        <v>0</v>
+        <v>14000</v>
       </c>
       <c r="G6" t="n">
         <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>0</v>
+        <v>14800</v>
       </c>
       <c r="I6" t="n">
-        <v>2900</v>
+        <v>-800</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2024-12</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>invoices</t>
-        </is>
+          <t>2025-04</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>14000</v>
       </c>
       <c r="C7" t="n">
-        <v>73200</v>
+        <v>77850</v>
       </c>
       <c r="D7" t="n">
-        <v>0</v>
+        <v>79850</v>
       </c>
       <c r="E7" t="n">
-        <v>0</v>
+        <v>12000</v>
       </c>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>12000</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>0</v>
+        <v>12800</v>
       </c>
       <c r="I7" t="n">
-        <v>73200</v>
+        <v>-800</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2024-12</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>schedule</t>
-        </is>
+          <t>2025-05</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>12000</v>
       </c>
       <c r="C8" t="n">
-        <v>75800</v>
+        <v>76150</v>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>78150</v>
       </c>
       <c r="E8" t="n">
-        <v>0</v>
+        <v>10000</v>
       </c>
       <c r="F8" t="n">
-        <v>0</v>
+        <v>10000</v>
       </c>
       <c r="G8" t="n">
         <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>0</v>
+        <v>10800</v>
       </c>
       <c r="I8" t="n">
-        <v>75800</v>
+        <v>-800</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2024-12</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>supported</t>
-        </is>
+          <t>2025-06</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>10000</v>
       </c>
       <c r="C9" t="n">
-        <v>72900</v>
+        <v>70250</v>
       </c>
       <c r="D9" t="n">
-        <v>0</v>
+        <v>75250</v>
       </c>
       <c r="E9" t="n">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="F9" t="n">
-        <v>0</v>
+        <v>8000</v>
       </c>
       <c r="G9" t="n">
-        <v>0</v>
+        <v>3000</v>
       </c>
       <c r="H9" t="n">
-        <v>0</v>
+        <v>5800</v>
       </c>
       <c r="I9" t="n">
-        <v>72900</v>
+        <v>-800</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2025-01</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>difference</t>
-        </is>
+          <t>2025-07</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>5000</v>
       </c>
       <c r="C10" t="n">
-        <v>2900</v>
+        <v>73150</v>
       </c>
       <c r="D10" t="n">
-        <v>4000</v>
+        <v>72150</v>
       </c>
       <c r="E10" t="n">
-        <v>0</v>
+        <v>6000</v>
       </c>
       <c r="F10" t="n">
-        <v>0</v>
+        <v>6000</v>
       </c>
       <c r="G10" t="n">
         <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>0</v>
+        <v>6800</v>
       </c>
       <c r="I10" t="n">
-        <v>6900</v>
+        <v>-800</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2025-01</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>invoices</t>
-        </is>
+          <t>2025-08</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>6000</v>
       </c>
       <c r="C11" t="n">
-        <v>73200</v>
+        <v>70150</v>
       </c>
       <c r="D11" t="n">
+        <v>72150</v>
+      </c>
+      <c r="E11" t="n">
         <v>4000</v>
       </c>
-      <c r="E11" t="n">
-        <v>0</v>
-      </c>
       <c r="F11" t="n">
-        <v>0</v>
+        <v>4000</v>
       </c>
       <c r="G11" t="n">
         <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>0</v>
+        <v>4800</v>
       </c>
       <c r="I11" t="n">
-        <v>77200</v>
+        <v>-800</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2025-01</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>schedule</t>
-        </is>
+          <t>2025-09</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>4000</v>
       </c>
       <c r="C12" t="n">
-        <v>75800</v>
+        <v>70150</v>
       </c>
       <c r="D12" t="n">
-        <v>8000</v>
+        <v>72150</v>
       </c>
       <c r="E12" t="n">
-        <v>0</v>
+        <v>2000</v>
       </c>
       <c r="F12" t="n">
-        <v>0</v>
+        <v>2000</v>
       </c>
       <c r="G12" t="n">
         <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>0</v>
+        <v>2800</v>
       </c>
       <c r="I12" t="n">
-        <v>83800</v>
+        <v>-800</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2025-01</t>
+          <t>2025-10</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>2000</v>
+      </c>
+      <c r="C13" t="n">
+        <v>70150</v>
+      </c>
+      <c r="D13" t="n">
+        <v>72150</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" t="n">
+        <v>800</v>
+      </c>
+      <c r="I13" t="n">
+        <v>-800</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E43"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>key</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>customer_name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>closing_deferred</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>closing_unbilled</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>months_of_deferred_cover</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>F-001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Blue Harbor Analytics</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>F-002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Granite Peak Software</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>F-003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Cedar Loop Systems</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>F-004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Northwind Dynamics</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>F-005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Juniper Ridge Labs</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>F-008</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Maple Street Health</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>F-009</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Lantern Field Co</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>F-010</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Copperline Freight</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>F-011</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Harbor Light Media</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>F-012</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Quiet Creek Software</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>F-013</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Fictional Co 13</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>F-014</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>supported</t>
+          <t>Fictional Co 14</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>72900</v>
+        <v>0</v>
       </c>
       <c r="D13" t="n">
-        <v>4000</v>
-      </c>
-      <c r="E13" t="n">
-        <v>0</v>
-      </c>
-      <c r="F13" t="n">
-        <v>0</v>
-      </c>
-      <c r="G13" t="n">
-        <v>0</v>
-      </c>
-      <c r="H13" t="n">
-        <v>0</v>
-      </c>
-      <c r="I13" t="n">
-        <v>76900</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="E13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2025-02</t>
+          <t>F-015</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>difference</t>
+          <t>Fictional Co 15</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>6900</v>
+        <v>0</v>
       </c>
       <c r="D14" t="n">
         <v>0</v>
       </c>
-      <c r="E14" t="n">
-        <v>0</v>
-      </c>
-      <c r="F14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G14" t="n">
-        <v>0</v>
-      </c>
-      <c r="H14" t="n">
-        <v>0</v>
-      </c>
-      <c r="I14" t="n">
-        <v>6900</v>
-      </c>
+      <c r="E14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2025-02</t>
+          <t>F-016</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>invoices</t>
+          <t>Fictional Co 16</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>77200</v>
+        <v>0</v>
       </c>
       <c r="D15" t="n">
-        <v>950</v>
-      </c>
-      <c r="E15" t="n">
-        <v>0</v>
-      </c>
-      <c r="F15" t="n">
-        <v>0</v>
-      </c>
-      <c r="G15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H15" t="n">
-        <v>0</v>
-      </c>
-      <c r="I15" t="n">
-        <v>78150</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="E15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2025-02</t>
+          <t>F-017</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>schedule</t>
+          <t>Fictional Co 17</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>83800</v>
+        <v>0</v>
       </c>
       <c r="D16" t="n">
         <v>0</v>
       </c>
-      <c r="E16" t="n">
-        <v>0</v>
-      </c>
-      <c r="F16" t="n">
-        <v>0</v>
-      </c>
-      <c r="G16" t="n">
-        <v>0</v>
-      </c>
-      <c r="H16" t="n">
-        <v>0</v>
-      </c>
-      <c r="I16" t="n">
-        <v>83800</v>
-      </c>
+      <c r="E16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2025-02</t>
+          <t>F-018</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>supported</t>
+          <t>Fictional Co 18</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>76900</v>
+        <v>0</v>
       </c>
       <c r="D17" t="n">
         <v>0</v>
       </c>
-      <c r="E17" t="n">
-        <v>0</v>
-      </c>
-      <c r="F17" t="n">
-        <v>0</v>
-      </c>
-      <c r="G17" t="n">
-        <v>0</v>
-      </c>
-      <c r="H17" t="n">
-        <v>0</v>
-      </c>
-      <c r="I17" t="n">
-        <v>76900</v>
-      </c>
+      <c r="E17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2025-03</t>
+          <t>F-019</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>difference</t>
+          <t>Fictional Co 19</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>6900</v>
+        <v>0</v>
       </c>
       <c r="D18" t="n">
         <v>0</v>
       </c>
-      <c r="E18" t="n">
-        <v>0</v>
-      </c>
-      <c r="F18" t="n">
-        <v>0</v>
-      </c>
-      <c r="G18" t="n">
-        <v>0</v>
-      </c>
-      <c r="H18" t="n">
-        <v>0</v>
-      </c>
-      <c r="I18" t="n">
-        <v>6900</v>
-      </c>
+      <c r="E18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2025-03</t>
+          <t>F-020</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>invoices</t>
+          <t>Fictional Co 20</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>78150</v>
+        <v>0</v>
       </c>
       <c r="D19" t="n">
         <v>0</v>
       </c>
-      <c r="E19" t="n">
-        <v>0</v>
-      </c>
-      <c r="F19" t="n">
-        <v>0</v>
-      </c>
-      <c r="G19" t="n">
-        <v>0</v>
-      </c>
-      <c r="H19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I19" t="n">
-        <v>78150</v>
-      </c>
+      <c r="E19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2025-03</t>
+          <t>F-021</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>schedule</t>
+          <t>Fictional Co 21</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>83800</v>
+        <v>0</v>
       </c>
       <c r="D20" t="n">
         <v>0</v>
       </c>
-      <c r="E20" t="n">
-        <v>0</v>
-      </c>
-      <c r="F20" t="n">
-        <v>0</v>
-      </c>
-      <c r="G20" t="n">
-        <v>0</v>
-      </c>
-      <c r="H20" t="n">
-        <v>0</v>
-      </c>
-      <c r="I20" t="n">
-        <v>83800</v>
-      </c>
+      <c r="E20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2025-03</t>
+          <t>F-022</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>supported</t>
+          <t>Fictional Co 22</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>76900</v>
+        <v>0</v>
       </c>
       <c r="D21" t="n">
         <v>0</v>
       </c>
-      <c r="E21" t="n">
-        <v>0</v>
-      </c>
-      <c r="F21" t="n">
-        <v>0</v>
-      </c>
-      <c r="G21" t="n">
-        <v>0</v>
-      </c>
-      <c r="H21" t="n">
-        <v>0</v>
-      </c>
-      <c r="I21" t="n">
-        <v>76900</v>
-      </c>
+      <c r="E21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2025-04</t>
+          <t>F-023</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>difference</t>
+          <t>Fictional Co 23</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>6900</v>
+        <v>0</v>
       </c>
       <c r="D22" t="n">
         <v>0</v>
       </c>
-      <c r="E22" t="n">
-        <v>0</v>
-      </c>
-      <c r="F22" t="n">
-        <v>-4000</v>
-      </c>
-      <c r="G22" t="n">
-        <v>0</v>
-      </c>
-      <c r="H22" t="n">
-        <v>0</v>
-      </c>
-      <c r="I22" t="n">
-        <v>2900</v>
-      </c>
+      <c r="E22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2025-04</t>
+          <t>F-024</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>invoices</t>
+          <t>Fictional Co 24</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>78150</v>
+        <v>0</v>
       </c>
       <c r="D23" t="n">
         <v>0</v>
       </c>
-      <c r="E23" t="n">
-        <v>0</v>
-      </c>
-      <c r="F23" t="n">
-        <v>5700</v>
-      </c>
-      <c r="G23" t="n">
-        <v>0</v>
-      </c>
-      <c r="H23" t="n">
-        <v>4000</v>
-      </c>
-      <c r="I23" t="n">
-        <v>79850</v>
-      </c>
+      <c r="E23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2025-04</t>
+          <t>F-025</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>schedule</t>
+          <t>Fictional Co 25</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>83800</v>
+        <v>0</v>
       </c>
       <c r="D24" t="n">
         <v>0</v>
       </c>
-      <c r="E24" t="n">
-        <v>0</v>
-      </c>
-      <c r="F24" t="n">
-        <v>0</v>
-      </c>
-      <c r="G24" t="n">
-        <v>0</v>
-      </c>
-      <c r="H24" t="n">
-        <v>4000</v>
-      </c>
-      <c r="I24" t="n">
-        <v>79800</v>
-      </c>
+      <c r="E24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2025-04</t>
+          <t>F-026</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>supported</t>
+          <t>Fictional Co 26</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>76900</v>
+        <v>0</v>
       </c>
       <c r="D25" t="n">
         <v>0</v>
       </c>
-      <c r="E25" t="n">
-        <v>0</v>
-      </c>
-      <c r="F25" t="n">
-        <v>4000</v>
-      </c>
-      <c r="G25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H25" t="n">
-        <v>4000</v>
-      </c>
-      <c r="I25" t="n">
-        <v>76900</v>
-      </c>
+      <c r="E25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2025-05</t>
+          <t>F-027</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>difference</t>
+          <t>Fictional Co 27</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>2900</v>
+        <v>0</v>
       </c>
       <c r="D26" t="n">
         <v>0</v>
       </c>
-      <c r="E26" t="n">
-        <v>0</v>
-      </c>
-      <c r="F26" t="n">
-        <v>0</v>
-      </c>
-      <c r="G26" t="n">
-        <v>0</v>
-      </c>
-      <c r="H26" t="n">
-        <v>0</v>
-      </c>
-      <c r="I26" t="n">
-        <v>2900</v>
-      </c>
+      <c r="E26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2025-05</t>
+          <t>F-028</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>invoices</t>
+          <t>Fictional Co 28</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>79850</v>
+        <v>0</v>
       </c>
       <c r="D27" t="n">
         <v>0</v>
       </c>
-      <c r="E27" t="n">
-        <v>0</v>
-      </c>
-      <c r="F27" t="n">
-        <v>0</v>
-      </c>
-      <c r="G27" t="n">
-        <v>1700</v>
-      </c>
-      <c r="H27" t="n">
-        <v>0</v>
-      </c>
-      <c r="I27" t="n">
-        <v>78150</v>
-      </c>
+      <c r="E27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2025-05</t>
+          <t>F-029</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>schedule</t>
+          <t>Fictional Co 29</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>79800</v>
+        <v>0</v>
       </c>
       <c r="D28" t="n">
         <v>0</v>
       </c>
-      <c r="E28" t="n">
-        <v>0</v>
-      </c>
-      <c r="F28" t="n">
-        <v>600</v>
-      </c>
-      <c r="G28" t="n">
-        <v>0</v>
-      </c>
-      <c r="H28" t="n">
-        <v>0</v>
-      </c>
-      <c r="I28" t="n">
-        <v>80400</v>
-      </c>
+      <c r="E28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2025-05</t>
+          <t>F-030</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>supported</t>
+          <t>Fictional Co 30</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>76900</v>
+        <v>0</v>
       </c>
       <c r="D29" t="n">
         <v>0</v>
       </c>
-      <c r="E29" t="n">
-        <v>0</v>
-      </c>
-      <c r="F29" t="n">
-        <v>600</v>
-      </c>
-      <c r="G29" t="n">
-        <v>0</v>
-      </c>
-      <c r="H29" t="n">
-        <v>0</v>
-      </c>
-      <c r="I29" t="n">
-        <v>77500</v>
-      </c>
+      <c r="E29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2025-06</t>
+          <t>F-031</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>difference</t>
+          <t>Fictional Co 31</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>2900</v>
+        <v>0</v>
       </c>
       <c r="D30" t="n">
         <v>0</v>
       </c>
-      <c r="E30" t="n">
-        <v>0</v>
-      </c>
-      <c r="F30" t="n">
-        <v>0</v>
-      </c>
-      <c r="G30" t="n">
-        <v>0</v>
-      </c>
-      <c r="H30" t="n">
-        <v>0</v>
-      </c>
-      <c r="I30" t="n">
-        <v>2900</v>
-      </c>
+      <c r="E30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2025-06</t>
+          <t>F-032</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>invoices</t>
+          <t>Fictional Co 32</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>78150</v>
+        <v>0</v>
       </c>
       <c r="D31" t="n">
         <v>0</v>
       </c>
-      <c r="E31" t="n">
-        <v>0</v>
-      </c>
-      <c r="F31" t="n">
-        <v>600</v>
-      </c>
-      <c r="G31" t="n">
-        <v>400</v>
-      </c>
-      <c r="H31" t="n">
-        <v>3100</v>
-      </c>
-      <c r="I31" t="n">
-        <v>75250</v>
-      </c>
+      <c r="E31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2025-06</t>
+          <t>F-033</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>schedule</t>
+          <t>Fictional Co 33</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>80400</v>
+        <v>0</v>
       </c>
       <c r="D32" t="n">
         <v>0</v>
       </c>
-      <c r="E32" t="n">
-        <v>0</v>
-      </c>
-      <c r="F32" t="n">
-        <v>0</v>
-      </c>
-      <c r="G32" t="n">
-        <v>400</v>
-      </c>
-      <c r="H32" t="n">
-        <v>3100</v>
-      </c>
-      <c r="I32" t="n">
-        <v>76900</v>
-      </c>
+      <c r="E32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2025-06</t>
+          <t>F-034</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>supported</t>
+          <t>Fictional Co 34</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>77500</v>
+        <v>0</v>
       </c>
       <c r="D33" t="n">
         <v>0</v>
       </c>
-      <c r="E33" t="n">
-        <v>0</v>
-      </c>
-      <c r="F33" t="n">
-        <v>0</v>
-      </c>
-      <c r="G33" t="n">
-        <v>400</v>
-      </c>
-      <c r="H33" t="n">
-        <v>3100</v>
-      </c>
-      <c r="I33" t="n">
-        <v>74000</v>
-      </c>
+      <c r="E33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2025-07</t>
+          <t>F-035</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>difference</t>
+          <t>Fictional Co 35</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>2900</v>
+        <v>0</v>
       </c>
       <c r="D34" t="n">
         <v>0</v>
       </c>
-      <c r="E34" t="n">
-        <v>0</v>
-      </c>
-      <c r="F34" t="n">
-        <v>0</v>
-      </c>
-      <c r="G34" t="n">
-        <v>0</v>
-      </c>
-      <c r="H34" t="n">
-        <v>0</v>
-      </c>
-      <c r="I34" t="n">
-        <v>2900</v>
-      </c>
+      <c r="E34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2025-07</t>
+          <t>F-036</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>invoices</t>
+          <t>Fictional Co 36</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>75250</v>
+        <v>0</v>
       </c>
       <c r="D35" t="n">
         <v>0</v>
       </c>
-      <c r="E35" t="n">
-        <v>0</v>
-      </c>
-      <c r="F35" t="n">
-        <v>0</v>
-      </c>
-      <c r="G35" t="n">
-        <v>0</v>
-      </c>
-      <c r="H35" t="n">
-        <v>3100</v>
-      </c>
-      <c r="I35" t="n">
-        <v>72150</v>
-      </c>
+      <c r="E35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2025-07</t>
+          <t>F-037</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>schedule</t>
+          <t>Fictional Co 37</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>76900</v>
+        <v>0</v>
       </c>
       <c r="D36" t="n">
         <v>0</v>
       </c>
-      <c r="E36" t="n">
-        <v>0</v>
-      </c>
-      <c r="F36" t="n">
-        <v>0</v>
-      </c>
-      <c r="G36" t="n">
-        <v>0</v>
-      </c>
-      <c r="H36" t="n">
-        <v>3100</v>
-      </c>
-      <c r="I36" t="n">
-        <v>73800</v>
-      </c>
+      <c r="E36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2025-07</t>
+          <t>F-038</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>supported</t>
+          <t>Fictional Co 38</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>74000</v>
+        <v>0</v>
       </c>
       <c r="D37" t="n">
         <v>0</v>
       </c>
-      <c r="E37" t="n">
-        <v>0</v>
-      </c>
-      <c r="F37" t="n">
-        <v>0</v>
-      </c>
-      <c r="G37" t="n">
-        <v>0</v>
-      </c>
-      <c r="H37" t="n">
-        <v>3100</v>
-      </c>
-      <c r="I37" t="n">
-        <v>70900</v>
-      </c>
+      <c r="E37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2025-08</t>
+          <t>F-039</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>difference</t>
+          <t>Fictional Co 39</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>2900</v>
+        <v>0</v>
       </c>
       <c r="D38" t="n">
         <v>0</v>
       </c>
-      <c r="E38" t="n">
-        <v>0</v>
-      </c>
-      <c r="F38" t="n">
-        <v>0</v>
-      </c>
-      <c r="G38" t="n">
-        <v>0</v>
-      </c>
-      <c r="H38" t="n">
-        <v>0</v>
-      </c>
-      <c r="I38" t="n">
-        <v>2900</v>
-      </c>
+      <c r="E38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2025-08</t>
+          <t>F-040</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>invoices</t>
+          <t>Fictional Co 40</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>72150</v>
+        <v>0</v>
       </c>
       <c r="D39" t="n">
         <v>0</v>
       </c>
-      <c r="E39" t="n">
-        <v>0</v>
-      </c>
-      <c r="F39" t="n">
-        <v>0</v>
-      </c>
-      <c r="G39" t="n">
-        <v>0</v>
-      </c>
-      <c r="H39" t="n">
-        <v>0</v>
-      </c>
-      <c r="I39" t="n">
-        <v>72150</v>
-      </c>
+      <c r="E39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2025-08</t>
+          <t>F-041</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>schedule</t>
+          <t>Fictional Co 41</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>73800</v>
+        <v>0</v>
       </c>
       <c r="D40" t="n">
         <v>0</v>
       </c>
-      <c r="E40" t="n">
-        <v>0</v>
-      </c>
-      <c r="F40" t="n">
-        <v>0</v>
-      </c>
-      <c r="G40" t="n">
-        <v>0</v>
-      </c>
-      <c r="H40" t="n">
-        <v>0</v>
-      </c>
-      <c r="I40" t="n">
-        <v>73800</v>
-      </c>
+      <c r="E40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2025-08</t>
+          <t>F-042</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>supported</t>
+          <t>Fictional Co 42</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>70900</v>
+        <v>0</v>
       </c>
       <c r="D41" t="n">
         <v>0</v>
       </c>
-      <c r="E41" t="n">
-        <v>0</v>
-      </c>
-      <c r="F41" t="n">
-        <v>0</v>
-      </c>
-      <c r="G41" t="n">
-        <v>0</v>
-      </c>
-      <c r="H41" t="n">
-        <v>0</v>
-      </c>
-      <c r="I41" t="n">
-        <v>70900</v>
-      </c>
+      <c r="E41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2025-09</t>
+          <t>INV-ONLY-1</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>difference</t>
+          <t>Orphan Billing LLC</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>2900</v>
+        <v>0</v>
       </c>
       <c r="D42" t="n">
         <v>0</v>
       </c>
-      <c r="E42" t="n">
-        <v>0</v>
-      </c>
-      <c r="F42" t="n">
-        <v>0</v>
-      </c>
-      <c r="G42" t="n">
-        <v>0</v>
-      </c>
-      <c r="H42" t="n">
-        <v>0</v>
-      </c>
-      <c r="I42" t="n">
-        <v>2900</v>
-      </c>
+      <c r="E42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2025-09</t>
+          <t>NAME:acme</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>invoices</t>
+          <t>ACME Corporation</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>72150</v>
+        <v>0</v>
       </c>
       <c r="D43" t="n">
         <v>0</v>
       </c>
-      <c r="E43" t="n">
-        <v>0</v>
-      </c>
-      <c r="F43" t="n">
-        <v>0</v>
-      </c>
-      <c r="G43" t="n">
-        <v>0</v>
-      </c>
-      <c r="H43" t="n">
-        <v>0</v>
-      </c>
-      <c r="I43" t="n">
-        <v>72150</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>2025-09</t>
-        </is>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>schedule</t>
-        </is>
-      </c>
-      <c r="C44" t="n">
-        <v>73800</v>
-      </c>
-      <c r="D44" t="n">
-        <v>0</v>
-      </c>
-      <c r="E44" t="n">
-        <v>0</v>
-      </c>
-      <c r="F44" t="n">
-        <v>0</v>
-      </c>
-      <c r="G44" t="n">
-        <v>0</v>
-      </c>
-      <c r="H44" t="n">
-        <v>1400</v>
-      </c>
-      <c r="I44" t="n">
-        <v>72400</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>2025-09</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>supported</t>
-        </is>
-      </c>
-      <c r="C45" t="n">
-        <v>70900</v>
-      </c>
-      <c r="D45" t="n">
-        <v>0</v>
-      </c>
-      <c r="E45" t="n">
-        <v>0</v>
-      </c>
-      <c r="F45" t="n">
-        <v>0</v>
-      </c>
-      <c r="G45" t="n">
-        <v>0</v>
-      </c>
-      <c r="H45" t="n">
-        <v>1400</v>
-      </c>
-      <c r="I45" t="n">
-        <v>69500</v>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>2025-10</t>
-        </is>
-      </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>difference</t>
-        </is>
-      </c>
-      <c r="C46" t="n">
-        <v>2900</v>
-      </c>
-      <c r="D46" t="n">
-        <v>0</v>
-      </c>
-      <c r="E46" t="n">
-        <v>0</v>
-      </c>
-      <c r="F46" t="n">
-        <v>0</v>
-      </c>
-      <c r="G46" t="n">
-        <v>0</v>
-      </c>
-      <c r="H46" t="n">
-        <v>0</v>
-      </c>
-      <c r="I46" t="n">
-        <v>2900</v>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>2025-10</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>invoices</t>
-        </is>
-      </c>
-      <c r="C47" t="n">
-        <v>72150</v>
-      </c>
-      <c r="D47" t="n">
-        <v>0</v>
-      </c>
-      <c r="E47" t="n">
-        <v>0</v>
-      </c>
-      <c r="F47" t="n">
-        <v>0</v>
-      </c>
-      <c r="G47" t="n">
-        <v>0</v>
-      </c>
-      <c r="H47" t="n">
-        <v>0</v>
-      </c>
-      <c r="I47" t="n">
-        <v>72150</v>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>2025-10</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>schedule</t>
-        </is>
-      </c>
-      <c r="C48" t="n">
-        <v>72400</v>
-      </c>
-      <c r="D48" t="n">
-        <v>0</v>
-      </c>
-      <c r="E48" t="n">
-        <v>0</v>
-      </c>
-      <c r="F48" t="n">
-        <v>0</v>
-      </c>
-      <c r="G48" t="n">
-        <v>0</v>
-      </c>
-      <c r="H48" t="n">
-        <v>0</v>
-      </c>
-      <c r="I48" t="n">
-        <v>72400</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>2025-10</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>supported</t>
-        </is>
-      </c>
-      <c r="C49" t="n">
-        <v>69500</v>
-      </c>
-      <c r="D49" t="n">
-        <v>0</v>
-      </c>
-      <c r="E49" t="n">
-        <v>0</v>
-      </c>
-      <c r="F49" t="n">
-        <v>0</v>
-      </c>
-      <c r="G49" t="n">
-        <v>0</v>
-      </c>
-      <c r="H49" t="n">
-        <v>0</v>
-      </c>
-      <c r="I49" t="n">
-        <v>69500</v>
-      </c>
+      <c r="E43" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>